<commit_message>
Fix UAT file headers and add the printable UAT plan
The UAT files kept the sample header (Grade 4 - Mabini, English,
2026-2027), which raised header warnings on upload to Rizal. They now say
Grade 6 - Rizal, Mathematics, 2025-2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/UAT-files/TC-022_valid-ecr-rizal.xlsx
+++ b/03-Testing/UAT-files/TC-022_valid-ecr-rizal.xlsx
@@ -13,11 +13,11 @@
     <sheet name="LRN" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'INPUT'!B11:B112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SUMMARY OF GRADES'!B12:B113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TERM1'!B11:B112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TERM2'!B11:B112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TERM3'!B11:B112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">INPUT!$B$11:$B$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'SUMMARY OF GRADES'!$B$12:$B$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">TERM1!$B$11:$B$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TERM2!$B$11:$B$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">TERM3!$B$11:$B$112</definedName>
     <definedName name="DESCRIPTORS">'Helper (Do Not Delete)'!$T$3:$W$7</definedName>
     <definedName name="FemaleLearners">INPUT!$B$63:$B$112</definedName>
     <definedName name="MaleLearners">INPUT!$B$12:$B$61</definedName>
@@ -148,10 +148,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -183,10 +183,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -467,7 +467,7 @@
         <v>SCHOOL YEAR</v>
       </c>
       <c r="Y5" t="str">
-        <v>2026-2027</v>
+        <v>2025-2026</v>
       </c>
     </row>
     <row r="7">
@@ -475,19 +475,19 @@
         <v xml:space="preserve">GRADE &amp; SECTION: </v>
       </c>
       <c r="J7" t="str">
-        <v>Grade 4 - Mabini</v>
+        <v>Grade 6 - Rizal</v>
       </c>
       <c r="N7" t="str">
         <v>TEACHER:</v>
       </c>
       <c r="Q7" t="str">
-        <v>Maria Elena Santos</v>
+        <v>Vilma Jordan Pines</v>
       </c>
       <c r="W7" t="str">
         <v>SUBJECT:</v>
       </c>
       <c r="Y7" t="str">
-        <v>English</v>
+        <v>Mathematics</v>
       </c>
     </row>
     <row r="8">
@@ -38870,7 +38870,7 @@
         <v>PERFORMANCE TASKS</v>
       </c>
       <c r="D1" t="str" xml:space="preserve">
-        <v xml:space="preserve">Q._x000d_
+        <v xml:space="preserve">Q.
 ASSESS-MENT</v>
       </c>
       <c r="G1" t="str">

</xml_diff>